<commit_message>
refactor: update finance report structure and add chart generation
</commit_message>
<xml_diff>
--- a/docs/template/summary.xlsx
+++ b/docs/template/summary.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11211"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/restupriyono/Downloads/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC6274C4-3184-4548-9263-415D42EEF212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -32,219 +27,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={952B16D3-B9CB-5344-94E4-09DA14C8D996}</author>
-    <author>tc={6690882D-83AE-4F49-AEA3-359933E838B6}</author>
-    <author>tc={306182D7-635D-AE43-8391-AE8BAF008B64}</author>
-    <author>tc={ED23E3CF-0195-5348-A86D-AB6D663010FB}</author>
-    <author>tc={1926CF56-FAB1-9F4F-A7CD-8366012E27A0}</author>
-    <author>tc={95184178-802D-B345-B1D8-5375EB49E7A1}</author>
-    <author>tc={903E833A-88A4-5D46-A612-23C625415198}</author>
-    <author>tc={4F96DB87-518E-E142-97BF-31275CEDEA7B}</author>
-    <author>tc={52E9E1DA-300F-8D43-AC9C-B5053804AADA}</author>
-    <author>tc={8A48D25F-E8B1-8D42-B1AA-6E0624B6E93D}</author>
-    <author>tc={C5F13C2E-400B-9B4C-9226-88092E6A2E86}</author>
-    <author>tc={1A4FBA55-6B42-C846-9F63-4250D577F01A}</author>
-  </authors>
-  <commentList>
-    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    zramadhan
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C6" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    hanif
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C7" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    dewani
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C8" authorId="3" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    herlan
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C9" authorId="4" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    hasan
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C10" authorId="5" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    rahmat
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C11" authorId="6" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    fathir
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C12" authorId="7" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    sagara
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C13" authorId="8" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    alkahfi
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C14" authorId="9" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    mulya
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C15" authorId="10" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    daus
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C16" authorId="11" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    pilihan
-</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3358,7 +3140,6 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <legacyDrawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>